<commit_message>
cập nhật file từ máy cơ quan
</commit_message>
<xml_diff>
--- a/Hoc_caohoc/hoso_caohoc/CTDT.xlsx
+++ b/Hoc_caohoc/hoso_caohoc/CTDT.xlsx
@@ -5,18 +5,17 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thongtin_giayto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Realstate\AAADongA_skill\Hoc_caohoc\hoso_caohoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210"/>
   </bookViews>
   <sheets>
     <sheet name="CTDT" sheetId="1" r:id="rId1"/>
     <sheet name="DkyHKI" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="164">
   <si>
     <t>KHUNG CHƯƠNG TRÌNH ĐÀO TẠO TRÌNH ĐỘ THẠC SĨ</t>
   </si>
@@ -561,12 +560,45 @@
   <si>
     <t>https://dangky.tlu.edu.vn/</t>
   </si>
+  <si>
+    <r>
+      <t>Địa chỉ (Address):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Khu Xuân Ổ A, Phường Võ Cường, Bắc Ninh, Việt Nam</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Mã số thuế (Tax code):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 2300786187　　　　</t>
+    </r>
+  </si>
+  <si>
+    <t>Trường Đại học công nghệ Đông Á</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -681,6 +713,14 @@
       <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -838,7 +878,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -998,6 +1038,18 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1010,9 +1062,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1022,21 +1071,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1058,9 +1101,7 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1360,80 +1401,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" customHeight="1">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="57"/>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1">
-      <c r="A4" s="60"/>
-      <c r="B4" s="60"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
+      <c r="A4" s="64"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="62" t="s">
+      <c r="C5" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="64" t="s">
+      <c r="D5" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="64"/>
-      <c r="F5" s="61" t="s">
+      <c r="E5" s="67"/>
+      <c r="F5" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="61" t="s">
+      <c r="G5" s="59" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" ht="28.5">
-      <c r="A6" s="61"/>
-      <c r="B6" s="63"/>
-      <c r="C6" s="63"/>
+      <c r="A6" s="59"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
       <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -1523,13 +1564,13 @@
       <c r="A11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="67" t="s">
+      <c r="B11" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="67"/>
-      <c r="D11" s="67"/>
-      <c r="E11" s="67"/>
-      <c r="F11" s="67"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="60"/>
+      <c r="F11" s="60"/>
       <c r="G11" s="13" t="s">
         <v>26</v>
       </c>
@@ -1538,13 +1579,13 @@
       <c r="A12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="67" t="s">
+      <c r="B12" s="60" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="67"/>
-      <c r="D12" s="67"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="67"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="14">
         <v>9</v>
       </c>
@@ -1622,13 +1663,13 @@
       <c r="A16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="67" t="s">
+      <c r="B16" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
       <c r="G16" s="13" t="s">
         <v>39</v>
       </c>
@@ -1867,13 +1908,13 @@
       <c r="A27" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="67" t="s">
+      <c r="B27" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="67"/>
-      <c r="D27" s="67"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="67"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="60"/>
       <c r="G27" s="14">
         <v>23</v>
       </c>
@@ -1882,13 +1923,13 @@
       <c r="A28" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="67" t="s">
+      <c r="B28" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="67"/>
-      <c r="D28" s="67"/>
-      <c r="E28" s="67"/>
-      <c r="F28" s="67"/>
+      <c r="C28" s="60"/>
+      <c r="D28" s="60"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="60"/>
       <c r="G28" s="14">
         <v>15</v>
       </c>
@@ -2012,13 +2053,13 @@
       <c r="A34" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="67" t="s">
+      <c r="B34" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="67"/>
-      <c r="D34" s="67"/>
-      <c r="E34" s="67"/>
-      <c r="F34" s="67"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="60"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="60"/>
       <c r="G34" s="14">
         <v>8</v>
       </c>
@@ -2202,24 +2243,24 @@
       </c>
     </row>
     <row r="43" spans="1:8" s="2" customFormat="1" ht="21" customHeight="1">
-      <c r="A43" s="61" t="s">
+      <c r="A43" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="B43" s="61"/>
-      <c r="C43" s="61"/>
-      <c r="D43" s="61"/>
-      <c r="E43" s="61"/>
-      <c r="F43" s="61"/>
+      <c r="B43" s="59"/>
+      <c r="C43" s="59"/>
+      <c r="D43" s="59"/>
+      <c r="E43" s="59"/>
+      <c r="F43" s="59"/>
       <c r="G43" s="14">
         <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="2" customFormat="1"/>
     <row r="45" spans="1:8" s="2" customFormat="1">
-      <c r="B45" s="65">
+      <c r="B45" s="57">
         <v>268119167</v>
       </c>
-      <c r="C45" s="66"/>
+      <c r="C45" s="58"/>
       <c r="D45" s="56" t="s">
         <v>112</v>
       </c>
@@ -2234,23 +2275,36 @@
       </c>
     </row>
     <row r="47" spans="1:8" s="2" customFormat="1"/>
-    <row r="48" spans="1:8" s="2" customFormat="1"/>
-    <row r="49" s="2" customFormat="1"/>
-    <row r="50" s="2" customFormat="1"/>
-    <row r="51" s="2" customFormat="1"/>
-    <row r="52" s="2" customFormat="1"/>
-    <row r="53" s="2" customFormat="1"/>
-    <row r="54" s="2" customFormat="1"/>
-    <row r="55" s="2" customFormat="1"/>
-    <row r="56" s="2" customFormat="1"/>
-    <row r="57" s="2" customFormat="1"/>
-    <row r="58" s="2" customFormat="1"/>
-    <row r="59" s="2" customFormat="1"/>
-    <row r="60" s="2" customFormat="1"/>
-    <row r="61" s="2" customFormat="1"/>
-    <row r="62" s="2" customFormat="1"/>
-    <row r="63" s="2" customFormat="1"/>
-    <row r="64" s="2" customFormat="1"/>
+    <row r="48" spans="1:8" s="2" customFormat="1">
+      <c r="B48" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C48" s="78" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3" s="2" customFormat="1">
+      <c r="C49"/>
+    </row>
+    <row r="50" spans="3:3" s="2" customFormat="1">
+      <c r="C50" s="78" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="51" spans="3:3" s="2" customFormat="1"/>
+    <row r="52" spans="3:3" s="2" customFormat="1"/>
+    <row r="53" spans="3:3" s="2" customFormat="1"/>
+    <row r="54" spans="3:3" s="2" customFormat="1"/>
+    <row r="55" spans="3:3" s="2" customFormat="1"/>
+    <row r="56" spans="3:3" s="2" customFormat="1"/>
+    <row r="57" spans="3:3" s="2" customFormat="1"/>
+    <row r="58" spans="3:3" s="2" customFormat="1"/>
+    <row r="59" spans="3:3" s="2" customFormat="1"/>
+    <row r="60" spans="3:3" s="2" customFormat="1"/>
+    <row r="61" spans="3:3" s="2" customFormat="1"/>
+    <row r="62" spans="3:3" s="2" customFormat="1"/>
+    <row r="63" spans="3:3" s="2" customFormat="1"/>
+    <row r="64" spans="3:3" s="2" customFormat="1"/>
     <row r="65" s="2" customFormat="1"/>
     <row r="66" s="2" customFormat="1"/>
     <row r="67" s="2" customFormat="1"/>
@@ -2289,14 +2343,6 @@
     <row r="100" s="2" customFormat="1"/>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B34:F34"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
@@ -2307,6 +2353,14 @@
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B34:F34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2356,10 +2410,10 @@
       <c r="H1" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="I1" s="70" t="s">
+      <c r="I1" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="J1" s="71"/>
+      <c r="J1" s="72"/>
       <c r="K1" s="28" t="s">
         <v>107</v>
       </c>
@@ -2374,7 +2428,7 @@
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="72" t="s">
+      <c r="A2" s="73" t="s">
         <v>111</v>
       </c>
       <c r="B2" s="32" t="s">
@@ -2416,7 +2470,7 @@
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="73"/>
+      <c r="A3" s="74"/>
       <c r="B3" s="32" t="s">
         <v>72</v>
       </c>
@@ -2458,7 +2512,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" ht="38.25" customHeight="1">
-      <c r="A4" s="73"/>
+      <c r="A4" s="74"/>
       <c r="B4" s="40" t="s">
         <v>20</v>
       </c>
@@ -2498,7 +2552,7 @@
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="73"/>
+      <c r="A5" s="74"/>
       <c r="B5" s="32" t="s">
         <v>58</v>
       </c>
@@ -2538,7 +2592,7 @@
       </c>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="73"/>
+      <c r="A6" s="74"/>
       <c r="B6" s="32" t="s">
         <v>29</v>
       </c>
@@ -2578,7 +2632,7 @@
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="73"/>
+      <c r="A7" s="74"/>
       <c r="B7" s="32" t="s">
         <v>32</v>
       </c>
@@ -2618,7 +2672,7 @@
       </c>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="73"/>
+      <c r="A8" s="74"/>
       <c r="B8" s="32" t="s">
         <v>68</v>
       </c>
@@ -2660,7 +2714,7 @@
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="73"/>
+      <c r="A9" s="74"/>
       <c r="B9" s="32" t="s">
         <v>74</v>
       </c>
@@ -2718,11 +2772,11 @@
       <c r="N10" s="45"/>
     </row>
     <row r="11" spans="1:14" ht="16.5" customHeight="1">
-      <c r="A11" s="74" t="s">
+      <c r="A11" s="75" t="s">
         <v>132</v>
       </c>
-      <c r="B11" s="74"/>
-      <c r="C11" s="74"/>
+      <c r="B11" s="75"/>
+      <c r="C11" s="75"/>
       <c r="D11" s="46"/>
       <c r="E11" s="47" t="s">
         <v>133</v>
@@ -2741,10 +2795,10 @@
       <c r="A12" s="48" t="s">
         <v>134</v>
       </c>
-      <c r="B12" s="75" t="s">
+      <c r="B12" s="76" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="76"/>
+      <c r="C12" s="77"/>
       <c r="D12" s="46"/>
       <c r="E12" s="49" t="s">
         <v>136</v>
@@ -2918,11 +2972,11 @@
       <c r="N18" s="46"/>
     </row>
     <row r="19" spans="1:14" ht="66" customHeight="1">
-      <c r="A19" s="77" t="s">
+      <c r="A19" s="70" t="s">
         <v>159</v>
       </c>
-      <c r="B19" s="77"/>
-      <c r="C19" s="77"/>
+      <c r="B19" s="70"/>
+      <c r="C19" s="70"/>
       <c r="D19" s="46"/>
       <c r="E19" s="46"/>
       <c r="F19" s="46"/>
@@ -2937,17 +2991,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="A19:C19"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="A2:A9"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A19:C19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>